<commit_message>
added exports and updated CAD's
</commit_message>
<xml_diff>
--- a/Electrical/PCB_Project/PCB_BOM.xlsx
+++ b/Electrical/PCB_Project/PCB_BOM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bryan Heddle\OneDrive\Desktop\Ergos-Dynamic-Humanoid-Platform\electrical\PCB_Project\Documents\Project Outputs for ROBOT_PCB_PROJECT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bryan Heddle\OneDrive\Desktop\Ergos-Dynamic-Humanoid-Platform\electrical\PCB_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99ED6EE7-F7E6-46F3-BBFC-6700AE5E11B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ACBB451-D29B-4522-993C-E998A3346260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{308192D4-E0FA-4898-8827-247AC0BD94FB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{308192D4-E0FA-4898-8827-247AC0BD94FB}"/>
   </bookViews>
   <sheets>
     <sheet name="AI_PCB_PROJECT" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="293">
   <si>
     <t>Line #</t>
   </si>
@@ -912,6 +912,12 @@
   </si>
   <si>
     <t>WM1399TR-ND</t>
+  </si>
+  <si>
+    <t>SN74LVC2G04DBVRG</t>
+  </si>
+  <si>
+    <t>RMCF0603FT47R0</t>
   </si>
 </sst>
 </file>
@@ -968,16 +974,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1317,11 +1322,11 @@
   <cols>
     <col min="1" max="1" width="9.28515625" customWidth="1"/>
     <col min="2" max="2" width="29.28515625" customWidth="1"/>
-    <col min="3" max="3" width="2.42578125" customWidth="1"/>
+    <col min="3" max="3" width="1.42578125" customWidth="1"/>
     <col min="4" max="4" width="26.42578125" customWidth="1"/>
-    <col min="5" max="5" width="2" customWidth="1"/>
+    <col min="5" max="5" width="1.140625" customWidth="1"/>
     <col min="6" max="6" width="11.28515625" customWidth="1"/>
-    <col min="7" max="7" width="16.85546875" customWidth="1"/>
+    <col min="7" max="7" width="31.140625" customWidth="1"/>
     <col min="8" max="8" width="27.42578125" customWidth="1"/>
     <col min="9" max="9" width="19.5703125" customWidth="1"/>
     <col min="10" max="10" width="19.28515625" customWidth="1"/>
@@ -1486,7 +1491,7 @@
       <c r="J4" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" t="s">
         <v>262</v>
       </c>
       <c r="L4" s="3">
@@ -1732,7 +1737,7 @@
       <c r="J10" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="K10" s="6" t="s">
+      <c r="K10" t="s">
         <v>263</v>
       </c>
       <c r="L10" s="3">
@@ -1894,7 +1899,7 @@
       <c r="J14" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="K14" s="6" t="s">
+      <c r="K14" t="s">
         <v>265</v>
       </c>
       <c r="L14" s="3">
@@ -2207,7 +2212,7 @@
       <c r="G22" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="H22" s="6" t="s">
+      <c r="H22" t="s">
         <v>277</v>
       </c>
       <c r="I22" s="3" t="s">
@@ -2216,7 +2221,7 @@
       <c r="J22" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="K22" s="6" t="s">
+      <c r="K22" t="s">
         <v>279</v>
       </c>
       <c r="L22" s="3">
@@ -2313,7 +2318,7 @@
         <v>147</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>148</v>
+        <v>292</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>149</v>
@@ -2667,7 +2672,7 @@
       <c r="J33" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="K33" s="6" t="s">
+      <c r="K33" t="s">
         <v>281</v>
       </c>
       <c r="L33" s="3">
@@ -2827,7 +2832,7 @@
       <c r="J37" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="K37" s="6" t="s">
+      <c r="K37" t="s">
         <v>284</v>
       </c>
       <c r="L37" s="3">
@@ -2907,7 +2912,7 @@
       <c r="J39" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="K39" s="6" t="s">
+      <c r="K39" t="s">
         <v>286</v>
       </c>
       <c r="L39" s="3">
@@ -2961,7 +2966,7 @@
         <v>235</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>236</v>
+        <v>291</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>237</v>

</xml_diff>